<commit_message>
Update ML algorithm results workbook
</commit_message>
<xml_diff>
--- a/Output of All ML Algo.xlsx
+++ b/Output of All ML Algo.xlsx
@@ -5,32 +5,22 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Class\Python Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Class\Python Project\ML-Algorithms-Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E986BC-95C1-4B12-8D2E-71BE5B868C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB534AA1-F897-4FD4-886E-1AB93F6A46E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{A016EB86-E396-4774-A5F6-6ED69BB50CF1}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Corrected Results" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Corrected Results'!$1:$2</definedName>
+  </definedNames>
+  <calcPr calcId="0"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -39,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="22">
   <si>
     <t>Name of Algorithms</t>
   </si>
@@ -75,13 +65,46 @@
   </si>
   <si>
     <t>Elastic Net</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Ridge Classifier</t>
+  </si>
+  <si>
+    <t>SGD Classifier</t>
+  </si>
+  <si>
+    <t>Note: Corrected multiclass classification results generated using training-only preprocessing.</t>
+  </si>
+  <si>
+    <t>Additional Comparison Metrics</t>
+  </si>
+  <si>
+    <t>0.2</t>
+  </si>
+  <si>
+    <t>0.4</t>
+  </si>
+  <si>
+    <t>0.6</t>
+  </si>
+  <si>
+    <t>Balanced accuracy</t>
+  </si>
+  <si>
+    <t>Macro-F1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -111,13 +134,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2F0D9"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="5">
@@ -135,19 +178,6 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -180,25 +210,65 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,25 +602,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{181F1154-0C5B-443B-8347-18608F6CA0BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" ht="23.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="6"/>
-      <c r="E1" s="7"/>
-    </row>
-    <row r="2" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="D1" s="10"/>
+      <c r="E1" s="11"/>
+    </row>
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2">
@@ -638,13 +708,13 @@
         <v>2</v>
       </c>
       <c r="C8" s="2">
-        <v>0.85350000000000004</v>
+        <v>0.98450000000000004</v>
       </c>
       <c r="D8" s="2">
-        <v>0.87450000000000006</v>
+        <v>0.98480000000000001</v>
       </c>
       <c r="E8" s="2">
-        <v>0.85829999999999995</v>
+        <v>0.98219999999999996</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -655,13 +725,13 @@
         <v>4</v>
       </c>
       <c r="C9" s="2">
-        <v>0.86860000000000004</v>
+        <v>0.98329999999999995</v>
       </c>
       <c r="D9" s="2">
-        <v>0.87450000000000006</v>
+        <v>0.98380000000000001</v>
       </c>
       <c r="E9" s="2">
-        <v>0.87360000000000004</v>
+        <v>0.98119999999999996</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -670,13 +740,13 @@
         <v>5</v>
       </c>
       <c r="C10" s="2">
-        <v>0.85350000000000004</v>
+        <v>0.98450000000000004</v>
       </c>
       <c r="D10" s="2">
-        <v>0.85470000000000002</v>
+        <v>0.98480000000000001</v>
       </c>
       <c r="E10" s="2">
-        <v>0.85829999999999995</v>
+        <v>0.98219999999999996</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -685,13 +755,13 @@
         <v>6</v>
       </c>
       <c r="C11" s="2">
-        <v>0.85489999999999999</v>
+        <v>0.98340000000000005</v>
       </c>
       <c r="D11" s="2">
-        <v>0.85419999999999996</v>
+        <v>0.98360000000000003</v>
       </c>
       <c r="E11" s="2">
-        <v>0.85960000000000003</v>
+        <v>0.98080000000000001</v>
       </c>
       <c r="H11" t="s">
         <v>8</v>
@@ -909,6 +979,231 @@
     <mergeCell ref="C1:E1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="5" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="D2" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="E2" s="5">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="7">
+        <v>0.76648611896285657</v>
+      </c>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="14"/>
+      <c r="B4" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="7">
+        <v>0.93511497762202078</v>
+      </c>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="14"/>
+      <c r="B5" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="7">
+        <v>0.76648611896285657</v>
+      </c>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="14"/>
+      <c r="B6" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="7">
+        <v>0.82413490737465911</v>
+      </c>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="7">
+        <v>0.9282303778514569</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="14"/>
+      <c r="B9" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="7">
+        <v>0.96436822380521026</v>
+      </c>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="14"/>
+      <c r="B10" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="7">
+        <v>0.9282303778514569</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="14"/>
+      <c r="B11" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="7">
+        <v>0.94335056735828304</v>
+      </c>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+    </row>
+    <row r="13" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="7">
+        <v>0.75105706757800528</v>
+      </c>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="14"/>
+      <c r="B18" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="7">
+        <v>0.3863859848595258</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="7">
+        <v>0.73688709792246776</v>
+      </c>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="14"/>
+      <c r="B21" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="7">
+        <v>0.50940943722442922</v>
+      </c>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A3:A6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update ML algorithm outputs and results
</commit_message>
<xml_diff>
--- a/Output of All ML Algo.xlsx
+++ b/Output of All ML Algo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Class\Python Project\ML-Algorithms-Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB534AA1-F897-4FD4-886E-1AB93F6A46E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BD00345-7BBC-47E2-AF27-C9097FA20168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -252,23 +252,23 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -639,13 +639,13 @@
         <v>2</v>
       </c>
       <c r="C3" s="2">
-        <v>0.93910000000000005</v>
+        <v>0.97050000000000003</v>
       </c>
       <c r="D3" s="2">
-        <v>0.93679999999999997</v>
+        <v>0.97430000000000005</v>
       </c>
       <c r="E3" s="2">
-        <v>0.92400000000000004</v>
+        <v>0.97829999999999995</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -656,13 +656,13 @@
         <v>4</v>
       </c>
       <c r="C4" s="2">
-        <v>0.93840000000000001</v>
+        <v>0.9657</v>
       </c>
       <c r="D4" s="2">
-        <v>0.93720000000000003</v>
+        <v>0.96960000000000002</v>
       </c>
       <c r="E4" s="2">
-        <v>0.93569999999999998</v>
+        <v>0.97330000000000005</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -671,13 +671,13 @@
         <v>5</v>
       </c>
       <c r="C5" s="2">
-        <v>0.93910000000000005</v>
+        <v>0.97050000000000003</v>
       </c>
       <c r="D5" s="2">
-        <v>0.93679999999999997</v>
+        <v>0.97430000000000005</v>
       </c>
       <c r="E5" s="2">
-        <v>0.92400000000000004</v>
+        <v>0.97829999999999995</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -686,13 +686,13 @@
         <v>6</v>
       </c>
       <c r="C6" s="2">
-        <v>0.93779999999999997</v>
+        <v>0.96789999999999998</v>
       </c>
       <c r="D6" s="2">
-        <v>0.93620000000000003</v>
+        <v>0.97170000000000001</v>
       </c>
       <c r="E6" s="2">
-        <v>0.92830000000000001</v>
+        <v>0.97560000000000002</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -780,13 +780,13 @@
         <v>2</v>
       </c>
       <c r="C13" s="2">
-        <v>0.74990000000000001</v>
+        <v>0.94489999999999996</v>
       </c>
       <c r="D13" s="2">
-        <v>0.75009999999999999</v>
+        <v>0.9446</v>
       </c>
       <c r="E13" s="2">
-        <v>0.75070000000000003</v>
+        <v>0.94499999999999995</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -797,13 +797,13 @@
         <v>4</v>
       </c>
       <c r="C14" s="2">
-        <v>0.96099999999999997</v>
+        <v>0.93330000000000002</v>
       </c>
       <c r="D14" s="2">
-        <v>0.96079999999999999</v>
+        <v>0.93279999999999996</v>
       </c>
       <c r="E14" s="2">
-        <v>0.96089999999999998</v>
+        <v>0.93340000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -812,13 +812,13 @@
         <v>5</v>
       </c>
       <c r="C15" s="2">
-        <v>0.74990000000000001</v>
+        <v>0.94489999999999996</v>
       </c>
       <c r="D15" s="2">
-        <v>0.75009999999999999</v>
+        <v>0.9446</v>
       </c>
       <c r="E15" s="2">
-        <v>0.75070000000000003</v>
+        <v>0.94499999999999995</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -827,13 +827,13 @@
         <v>6</v>
       </c>
       <c r="C16" s="2">
-        <v>0.83799999999999997</v>
+        <v>0.93579999999999997</v>
       </c>
       <c r="D16" s="2">
-        <v>0.83799999999999997</v>
+        <v>0.93559999999999999</v>
       </c>
       <c r="E16" s="2">
-        <v>0.83830000000000005</v>
+        <v>0.93600000000000005</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -849,13 +849,13 @@
         <v>2</v>
       </c>
       <c r="C18" s="2">
-        <v>0.75370000000000004</v>
+        <v>0.97199999999999998</v>
       </c>
       <c r="D18" s="2">
-        <v>0.75549999999999995</v>
+        <v>0.97240000000000004</v>
       </c>
       <c r="E18" s="2">
-        <v>0.75480000000000003</v>
+        <v>0.97699999999999998</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -866,13 +866,13 @@
         <v>4</v>
       </c>
       <c r="C19" s="2">
-        <v>0.95650000000000002</v>
+        <v>0.96689999999999998</v>
       </c>
       <c r="D19" s="2">
-        <v>0.95660000000000001</v>
+        <v>0.9677</v>
       </c>
       <c r="E19" s="2">
-        <v>0.95660000000000001</v>
+        <v>0.97209999999999996</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -881,13 +881,13 @@
         <v>5</v>
       </c>
       <c r="C20" s="2">
-        <v>0.75370000000000004</v>
+        <v>0.97199999999999998</v>
       </c>
       <c r="D20" s="2">
-        <v>0.75549999999999995</v>
+        <v>0.97240000000000004</v>
       </c>
       <c r="E20" s="2">
-        <v>0.75480000000000003</v>
+        <v>0.97699999999999998</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -896,13 +896,13 @@
         <v>6</v>
       </c>
       <c r="C21" s="2">
-        <v>0.83830000000000005</v>
+        <v>0.96919999999999995</v>
       </c>
       <c r="D21" s="2">
-        <v>0.83930000000000005</v>
+        <v>0.96970000000000001</v>
       </c>
       <c r="E21" s="2">
-        <v>0.83889999999999998</v>
+        <v>0.97450000000000003</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -918,13 +918,13 @@
         <v>2</v>
       </c>
       <c r="C23" s="2">
-        <v>0.753</v>
+        <v>0.96309999999999996</v>
       </c>
       <c r="D23" s="2">
-        <v>0.75429999999999997</v>
+        <v>0.96550000000000002</v>
       </c>
       <c r="E23" s="2">
-        <v>0.75370000000000004</v>
+        <v>0.96540000000000004</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
@@ -935,13 +935,13 @@
         <v>4</v>
       </c>
       <c r="C24" s="2">
-        <v>0.95650000000000002</v>
+        <v>0.95520000000000005</v>
       </c>
       <c r="D24" s="2">
-        <v>0.95660000000000001</v>
+        <v>0.95879999999999999</v>
       </c>
       <c r="E24" s="2">
-        <v>0.95660000000000001</v>
+        <v>0.9587</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -950,13 +950,13 @@
         <v>5</v>
       </c>
       <c r="C25" s="2">
-        <v>0.753</v>
+        <v>0.96309999999999996</v>
       </c>
       <c r="D25" s="2">
-        <v>0.75429999999999997</v>
+        <v>0.96550000000000002</v>
       </c>
       <c r="E25" s="2">
-        <v>0.75370000000000004</v>
+        <v>0.96540000000000004</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
@@ -965,13 +965,13 @@
         <v>6</v>
       </c>
       <c r="C26" s="2">
-        <v>0.83779999999999999</v>
+        <v>0.95850000000000002</v>
       </c>
       <c r="D26" s="2">
-        <v>0.83850000000000002</v>
+        <v>0.96160000000000001</v>
       </c>
       <c r="E26" s="2">
-        <v>0.83819999999999995</v>
+        <v>0.96150000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -1000,11 +1000,11 @@
       <c r="B1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
@@ -1020,7 +1020,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="6" t="s">
@@ -1033,7 +1033,7 @@
       <c r="E3" s="8"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="14"/>
+      <c r="A4" s="13"/>
       <c r="B4" s="6" t="s">
         <v>4</v>
       </c>
@@ -1044,7 +1044,7 @@
       <c r="E4" s="8"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="14"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="6" t="s">
         <v>5</v>
       </c>
@@ -1055,7 +1055,7 @@
       <c r="E5" s="8"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="14"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="6" t="s">
         <v>6</v>
       </c>
@@ -1066,7 +1066,7 @@
       <c r="E6" s="8"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="12" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -1079,7 +1079,7 @@
       <c r="E8" s="8"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="14"/>
+      <c r="A9" s="13"/>
       <c r="B9" s="6" t="s">
         <v>4</v>
       </c>
@@ -1090,7 +1090,7 @@
       <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
+      <c r="A10" s="13"/>
       <c r="B10" s="6" t="s">
         <v>5</v>
       </c>
@@ -1101,7 +1101,7 @@
       <c r="E10" s="8"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="14"/>
+      <c r="A11" s="13"/>
       <c r="B11" s="6" t="s">
         <v>6</v>
       </c>
@@ -1112,22 +1112,22 @@
       <c r="E11" s="8"/>
     </row>
     <row r="13" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
@@ -1147,7 +1147,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="12" t="s">
         <v>13</v>
       </c>
       <c r="B17" s="6" t="s">
@@ -1160,7 +1160,7 @@
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="14"/>
+      <c r="A18" s="13"/>
       <c r="B18" s="6" t="s">
         <v>21</v>
       </c>
@@ -1171,7 +1171,7 @@
       <c r="E18" s="8"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="12" t="s">
         <v>14</v>
       </c>
       <c r="B20" s="6" t="s">
@@ -1184,7 +1184,7 @@
       <c r="E20" s="8"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="14"/>
+      <c r="A21" s="13"/>
       <c r="B21" s="6" t="s">
         <v>21</v>
       </c>

</xml_diff>